<commit_message>
Boom-Bust-new time series form tyler 2010 ecological monographs: 8-21-2025
</commit_message>
<xml_diff>
--- a/data/BoomBust_Mechanisms.xlsx
+++ b/data/BoomBust_Mechanisms.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f4f5e485ed766aa2/Pictures/Documents/Career/Journal Publications/Manuscripts/Dissertation/boom-bust/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="327" documentId="8_{1B1AAC56-C345-4EC3-95A7-6FD9A5B02C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD805813-4E07-40B2-8E5C-BC5488B041BC}"/>
+  <xr:revisionPtr revIDLastSave="457" documentId="8_{1B1AAC56-C345-4EC3-95A7-6FD9A5B02C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EAB55474-0266-4454-828D-26802BD9B0BC}"/>
   <bookViews>
     <workbookView xWindow="-19320" yWindow="-60" windowWidth="19440" windowHeight="14880" activeTab="1" xr2:uid="{D0698BA0-D8A4-462B-B44D-ABAD27A63A84}"/>
   </bookViews>
@@ -17,7 +17,6 @@
     <sheet name="Mechanism" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="119">
   <si>
     <t>Paper</t>
   </si>
@@ -289,9 +288,6 @@
     <t>Mayaheros urophthalmus</t>
   </si>
   <si>
-    <t>Unfavorable environmental conditions</t>
-  </si>
-  <si>
     <t>1) After cold fronts, most sites saw declines in mayan cichlid numbers, the rest of the discussion and results were about the impacts of mayan cichlids on native communities.</t>
   </si>
   <si>
@@ -316,9 +312,6 @@
     <t>1) Abunances of cats increase 1-2 years after heavy rainfall years which coincides with large increases in small mammal abundance's</t>
   </si>
   <si>
-    <t>Resource matching from pulsed resource event</t>
-  </si>
-  <si>
     <t>The Budgerigar in Florida: Rise and Fall of an Exotic Psittacid</t>
   </si>
   <si>
@@ -328,9 +321,6 @@
     <t>Melopsittacus undulatus</t>
   </si>
   <si>
-    <t>Boom-bust</t>
-  </si>
-  <si>
     <t>1) Four extremely severe cold fronts occurred in 1977, 1983, 1986 and 1989, but there were no declines in abundance after the 3 of the 4 freezes, Cold alone is not a common driver of bird mortality, but lack of food from sudden freezes and snow cover are more common. the native habitat in australia udergos cold front of similar magnitude so they should be relatively resistant to the cold</t>
   </si>
   <si>
@@ -341,6 +331,69 @@
   </si>
   <si>
     <t>Poor*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Morris et al. </t>
+  </si>
+  <si>
+    <t>Using long-term datasets to study exotic plant invasions on rangelands in the western United States</t>
+  </si>
+  <si>
+    <t>Salsola tragus</t>
+  </si>
+  <si>
+    <t>1)It was inferred that since Lehmann lovegrass was shown to increase due to above average rainfall and then a subsequent drought that this was a similar mechanism for this species.</t>
+  </si>
+  <si>
+    <t>Environmental thresholds for pulsed resources</t>
+  </si>
+  <si>
+    <t>Contrasting invasion histories and effects of three non-native fishes observed with long-term monitoring data</t>
+  </si>
+  <si>
+    <t>Pintar et al.</t>
+  </si>
+  <si>
+    <t>Hemichromis letourneuxi</t>
+  </si>
+  <si>
+    <t>1) Cold water and drought events preceeded the boom-bust, and large non-native fishes experienced declines during those cold water conditions</t>
+  </si>
+  <si>
+    <t>2) Paper was more focused on impacts that non-natives have on native species</t>
+  </si>
+  <si>
+    <t>Environmental thresholds for ambient abiotic conditions</t>
+  </si>
+  <si>
+    <t>The Rise and Fall of a Reindeer Herd</t>
+  </si>
+  <si>
+    <t>Scheffer</t>
+  </si>
+  <si>
+    <t>Rangifer tarandus</t>
+  </si>
+  <si>
+    <t>1) There are no predators large enough to hunt reindeer in the islans</t>
+  </si>
+  <si>
+    <t>2) From behavioral observations and food preference experiments, taller shrub-like lichens are a key winter foods supply for the reindeer, a combination of cold winters that crusted ice inhibiting reindeer to access the lichens and large numbers that depleted the lichens, die offs were seen during the winter.</t>
+  </si>
+  <si>
+    <t>3) a small lack of sampling, corresponded with a period of military occupation, so poaching could have happened but the decline in popualtion size was already underway.</t>
+  </si>
+  <si>
+    <t>4) Disease and inbreeding were mentioned and ruled out, but with little rationale</t>
+  </si>
+  <si>
+    <t>Extreme Overshoot Of Resource Carrying Capacity</t>
+  </si>
+  <si>
+    <t>Intermediate</t>
+  </si>
+  <si>
+    <t>5) Question was why didn't St. George Island have a similar trend though the islands were of similar size</t>
   </si>
 </sst>
 </file>
@@ -414,18 +467,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -436,6 +477,18 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -795,7 +848,7 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
@@ -811,7 +864,7 @@
         <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
@@ -819,7 +872,7 @@
         <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -829,7 +882,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CF18FAA-193E-4ADD-BAC0-7E416D9C0956}">
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.5546875" customWidth="1"/>
@@ -838,7 +891,7 @@
     <col min="4" max="4" width="24.109375" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
     <col min="6" max="6" width="18.77734375" customWidth="1"/>
-    <col min="7" max="7" width="64.109375" customWidth="1"/>
+    <col min="7" max="7" width="67.6640625" customWidth="1"/>
     <col min="8" max="8" width="21.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="57.77734375" customWidth="1"/>
   </cols>
@@ -867,22 +920,22 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="11" t="s">
         <v>26</v>
       </c>
       <c r="G2" t="s">
@@ -890,33 +943,33 @@
       </c>
     </row>
     <row r="3" spans="1:7" ht="72" x14ac:dyDescent="0.3">
-      <c r="A3" s="5"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
+      <c r="A3" s="8"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
       <c r="G3" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="8" t="s">
         <v>78</v>
       </c>
       <c r="G4" s="1" t="s">
@@ -924,66 +977,66 @@
       </c>
     </row>
     <row r="5" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="5"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
+      <c r="A5" s="8"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
       <c r="G5" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="5"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
+      <c r="A6" s="8"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
       <c r="G6" s="1" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="5"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
       <c r="G7" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
+      <c r="A8" s="8"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
       <c r="G8" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="10" t="s">
         <v>79</v>
       </c>
       <c r="G9" s="1" t="s">
@@ -991,55 +1044,55 @@
       </c>
     </row>
     <row r="10" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="4"/>
+      <c r="A10" s="8"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="10"/>
       <c r="G10" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="5"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="4"/>
+      <c r="A11" s="8"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="10"/>
       <c r="G11" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="5"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="4"/>
+      <c r="A12" s="8"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="10"/>
       <c r="G12" s="1" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="10" t="s">
         <v>44</v>
       </c>
       <c r="G13" s="1" t="s">
@@ -1047,44 +1100,44 @@
       </c>
     </row>
     <row r="14" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="4"/>
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="10"/>
       <c r="G14" s="1" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="4"/>
+      <c r="A15" s="8"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="10"/>
       <c r="G15" s="1" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="E16" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="10" t="s">
         <v>44</v>
       </c>
       <c r="G16" s="1" t="s">
@@ -1092,56 +1145,56 @@
       </c>
     </row>
     <row r="17" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A17" s="5"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="4"/>
+      <c r="A17" s="8"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="10"/>
       <c r="G17" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="5"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="4"/>
+      <c r="A18" s="8"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="10"/>
       <c r="G18" s="1" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="5"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="4"/>
+      <c r="A19" s="8"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="10"/>
       <c r="G19" s="1" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="5"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="4"/>
+      <c r="A20" s="8"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="10"/>
       <c r="G20" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="5"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="4"/>
+      <c r="A21" s="8"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="10"/>
       <c r="G21" s="1" t="s">
         <v>50</v>
       </c>
@@ -1153,16 +1206,16 @@
       <c r="B22" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="E22" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F22" s="10" t="s">
+      <c r="F22" s="6" t="s">
         <v>54</v>
       </c>
       <c r="G22" s="1" t="s">
@@ -1173,19 +1226,19 @@
       <c r="A23" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E23" s="10" t="s">
+      <c r="E23" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F23" s="10" t="s">
+      <c r="F23" s="6" t="s">
         <v>54</v>
       </c>
       <c r="G23" s="1" t="s">
@@ -1193,22 +1246,22 @@
       </c>
     </row>
     <row r="24" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E24" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="10" t="s">
         <v>44</v>
       </c>
       <c r="G24" s="1" t="s">
@@ -1216,44 +1269,44 @@
       </c>
     </row>
     <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="4"/>
+      <c r="A25" s="8"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="10"/>
       <c r="G25" s="1" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A26" s="5"/>
-      <c r="B26" s="5"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="4"/>
+      <c r="A26" s="8"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="10"/>
       <c r="G26" s="1" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F27" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G27" s="1" t="s">
@@ -1261,12 +1314,12 @@
       </c>
     </row>
     <row r="28" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A28" s="5"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
+      <c r="A28" s="8"/>
+      <c r="B28" s="10"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="10"/>
       <c r="G28" s="1" t="s">
         <v>67</v>
       </c>
@@ -1275,103 +1328,233 @@
       <c r="A29" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D29" s="6" t="s">
         <v>14</v>
       </c>
       <c r="E29" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G29" s="4" t="s">
         <v>83</v>
-      </c>
-      <c r="F29" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="G29" s="8" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B30" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="C30" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="D30" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G30" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="D30" s="10" t="s">
+    </row>
+    <row r="31" spans="1:7" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D31" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E30" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="F30" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="G30" s="8" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B31" s="4" t="s">
+      <c r="E31" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="G31" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C31" s="6" t="s">
+    </row>
+    <row r="32" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A32" s="8"/>
+      <c r="B32" s="10"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D31" s="4" t="s">
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="8"/>
+      <c r="B33" s="10"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="E31" s="5" t="s">
+    </row>
+    <row r="34" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E35" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="F31" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="G31" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="5"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="6"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
-      <c r="G32" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" s="5"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="6"/>
-      <c r="D33" s="4"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
-      <c r="G33" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A34" s="8"/>
-      <c r="B34" s="10"/>
-      <c r="C34" s="11"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="8"/>
-      <c r="F34" s="8"/>
+      <c r="F35" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="8"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="F37" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A38" s="8"/>
+      <c r="B38" s="10"/>
+      <c r="C38" s="9"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A39" s="8"/>
+      <c r="B39" s="10"/>
+      <c r="C39" s="9"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A40" s="8"/>
+      <c r="B40" s="10"/>
+      <c r="C40" s="9"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A41" s="8"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="8"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="1" t="s">
+        <v>118</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="48">
+  <mergeCells count="60">
+    <mergeCell ref="F37:F41"/>
+    <mergeCell ref="E37:E41"/>
+    <mergeCell ref="D37:D41"/>
+    <mergeCell ref="C37:C41"/>
+    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="A37:A41"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="C35:C36"/>
     <mergeCell ref="F24:F26"/>
     <mergeCell ref="F27:F28"/>
     <mergeCell ref="A31:A33"/>
@@ -1380,46 +1563,44 @@
     <mergeCell ref="D31:D33"/>
     <mergeCell ref="E31:E33"/>
     <mergeCell ref="F31:F33"/>
+    <mergeCell ref="A16:A21"/>
+    <mergeCell ref="B16:B21"/>
+    <mergeCell ref="C16:C21"/>
+    <mergeCell ref="D16:D21"/>
+    <mergeCell ref="E16:E21"/>
+    <mergeCell ref="E9:E12"/>
+    <mergeCell ref="D9:D12"/>
+    <mergeCell ref="C9:C12"/>
+    <mergeCell ref="B9:B12"/>
+    <mergeCell ref="A9:A12"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="D13:D15"/>
+    <mergeCell ref="E13:E15"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="A4:A8"/>
+    <mergeCell ref="B4:B8"/>
+    <mergeCell ref="C4:C8"/>
+    <mergeCell ref="D4:D8"/>
+    <mergeCell ref="E4:E8"/>
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="F4:F8"/>
     <mergeCell ref="F9:F12"/>
     <mergeCell ref="F13:F15"/>
     <mergeCell ref="F16:F21"/>
+    <mergeCell ref="E24:E26"/>
+    <mergeCell ref="D24:D26"/>
+    <mergeCell ref="C24:C26"/>
     <mergeCell ref="A27:A28"/>
     <mergeCell ref="B27:B28"/>
     <mergeCell ref="C27:C28"/>
     <mergeCell ref="D27:D28"/>
     <mergeCell ref="E27:E28"/>
-    <mergeCell ref="A4:A8"/>
-    <mergeCell ref="B4:B8"/>
-    <mergeCell ref="C4:C8"/>
-    <mergeCell ref="D4:D8"/>
-    <mergeCell ref="E4:E8"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="D13:D15"/>
-    <mergeCell ref="E13:E15"/>
-    <mergeCell ref="E9:E12"/>
-    <mergeCell ref="D9:D12"/>
-    <mergeCell ref="C9:C12"/>
-    <mergeCell ref="B9:B12"/>
-    <mergeCell ref="A9:A12"/>
-    <mergeCell ref="A16:A21"/>
-    <mergeCell ref="B16:B21"/>
-    <mergeCell ref="C16:C21"/>
-    <mergeCell ref="D16:D21"/>
-    <mergeCell ref="E16:E21"/>
-    <mergeCell ref="E24:E26"/>
-    <mergeCell ref="D24:D26"/>
-    <mergeCell ref="C24:C26"/>
-    <mergeCell ref="B24:B26"/>
-    <mergeCell ref="A24:A26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Repository Clean Up: 9/2/2025
</commit_message>
<xml_diff>
--- a/data/BoomBust_Mechanisms.xlsx
+++ b/data/BoomBust_Mechanisms.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f4f5e485ed766aa2/Pictures/Documents/Career/Journal Publications/Manuscripts/Dissertation/boom-bust/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="472" documentId="8_{1B1AAC56-C345-4EC3-95A7-6FD9A5B02C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77DAC169-5DEF-4583-A30C-A98BC6EE9417}"/>
+  <xr:revisionPtr revIDLastSave="712" documentId="8_{1B1AAC56-C345-4EC3-95A7-6FD9A5B02C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B2152032-4CBD-4712-BE58-043CEFB140DC}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D0698BA0-D8A4-462B-B44D-ABAD27A63A84}"/>
+    <workbookView xWindow="-19320" yWindow="-60" windowWidth="19440" windowHeight="14880" activeTab="1" xr2:uid="{D0698BA0-D8A4-462B-B44D-ABAD27A63A84}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="2" r:id="rId1"/>
-    <sheet name="Mechanism" sheetId="1" r:id="rId2"/>
+    <sheet name="Mechanism_Supplementary" sheetId="1" r:id="rId2"/>
+    <sheet name="Table 1" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="128">
   <si>
     <t>Paper</t>
   </si>
@@ -138,9 +139,6 @@
     <t xml:space="preserve">1) Rock substrate is the preferable shelter from predation and cannabilism for rusty crayfish, but they can use macrophytes as well. </t>
   </si>
   <si>
-    <t>Invasive species unfavorabley alters ecosystem for future generations</t>
-  </si>
-  <si>
     <t>3) Presented data show a strong association between lakes that have declines like these lakes and lakes that had no declines and the prevalence of substrate. This is strong evidence because there was multiple lakes so larger sample size</t>
   </si>
   <si>
@@ -355,9 +353,6 @@
   </si>
   <si>
     <t>Hemichromis letourneuxi</t>
-  </si>
-  <si>
-    <t>1) Cold water and drought events preceeded the boom-bust, and large non-native fishes experienced declines during those cold water conditions</t>
   </si>
   <si>
     <t>2) Paper was more focused on impacts that non-natives have on native species</t>
@@ -421,12 +416,42 @@
   <si>
     <t>5) Total snowfall appeared to correlate with declines when presented, but there were counter examples, suggesting that there is a synergy between high numbers and high snow</t>
   </si>
+  <si>
+    <t>Invasive species unfavorabley alters ecosystem for future generations*</t>
+  </si>
+  <si>
+    <t>Number of Studies</t>
+  </si>
+  <si>
+    <t>Strong</t>
+  </si>
+  <si>
+    <t>Intermediate</t>
+  </si>
+  <si>
+    <t>Environmental Thresholds</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Invasive species unfavorably alter ecosystem for future generations</t>
+  </si>
+  <si>
+    <t>Not Specified</t>
+  </si>
+  <si>
+    <t>1) Cold water and drought events preceeded the boom-bust, and large non-native fishes experienced declines during those cold water conditions and drought conditions</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -442,6 +467,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -451,7 +484,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -479,11 +512,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="dotted">
+        <color theme="0" tint="-0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -504,6 +555,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -513,8 +567,78 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -874,7 +998,7 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
@@ -890,7 +1014,7 @@
         <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
@@ -898,7 +1022,7 @@
         <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -930,7 +1054,7 @@
         <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>13</v>
@@ -946,22 +1070,22 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="D2" s="8" t="s">
+      <c r="C2" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="D2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E2" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F2" s="8" t="s">
         <v>26</v>
       </c>
       <c r="G2" t="s">
@@ -969,294 +1093,294 @@
       </c>
     </row>
     <row r="3" spans="1:7" ht="72" x14ac:dyDescent="0.3">
-      <c r="A3" s="9"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
+      <c r="A3" s="10"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
       <c r="G3" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="D4" s="9" t="s">
+      <c r="C4" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="9" t="s">
-        <v>78</v>
+      <c r="F4" s="10" t="s">
+        <v>77</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
+      <c r="A5" s="10"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
       <c r="G5" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="9"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
+      <c r="A6" s="10"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
       <c r="G6" s="1" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
+      <c r="A7" s="10"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
       <c r="G7" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="9"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
+      <c r="A8" s="10"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
       <c r="G8" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D9" s="9" t="s">
+      <c r="C9" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>79</v>
+      <c r="E9" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>78</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="9"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="8"/>
+      <c r="A10" s="10"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="9"/>
       <c r="G10" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="10"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="10"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="9"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="9"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="1" t="s">
+    <row r="13" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="10" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="9" t="s">
+      <c r="B13" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="C13" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A14" s="10"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="10" t="s">
+    </row>
+    <row r="15" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D16" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E16" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F16" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="G16" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G13" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="9"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="9"/>
-      <c r="B15" s="9"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="G16" s="1" t="s">
+    </row>
+    <row r="17" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="10"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A17" s="9"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="1" t="s">
+    <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="10"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="9"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="1" t="s">
+    <row r="19" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A19" s="10"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="9"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="1" t="s">
+    <row r="20" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="10"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="9"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="1" t="s">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="10"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="1" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="9"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="C22" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D22" s="6" t="s">
         <v>52</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>53</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>27</v>
       </c>
       <c r="F22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G22" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>57</v>
-      </c>
       <c r="C23" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>14</v>
@@ -1265,347 +1389,313 @@
         <v>27</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G23" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A24" s="10" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="9" t="s">
+      <c r="B24" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="C24" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="G24" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C24" s="10" t="s">
+    </row>
+    <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="10"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A26" s="10"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C27" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="E24" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F24" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A25" s="9"/>
-      <c r="B25" s="9"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A26" s="9"/>
-      <c r="B26" s="9"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="8"/>
-      <c r="G26" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="B27" s="8" t="s">
+      <c r="D27" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G27" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C27" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="D27" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="F27" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="G27" s="1" t="s">
+    </row>
+    <row r="28" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="10"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="1" t="s">
         <v>66</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A28" s="9"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="62.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="C29" s="7" t="s">
         <v>81</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>14</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B30" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="C30" s="5" t="s">
         <v>88</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>89</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>14</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G30" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="10" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="9" t="s">
+      <c r="B31" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="C31" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="D31" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E31" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F31" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="G31" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="D31" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E31" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F31" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="G31" s="1" t="s">
+    </row>
+    <row r="32" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A32" s="10"/>
+      <c r="B32" s="9"/>
+      <c r="C32" s="11"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="9"/>
-      <c r="B32" s="8"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="9"/>
-      <c r="F32" s="9"/>
-      <c r="G32" s="1" t="s">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="10"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="11"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="1" t="s">
         <v>95</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" s="9"/>
-      <c r="B33" s="8"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="8"/>
-      <c r="E33" s="9"/>
-      <c r="F33" s="9"/>
-      <c r="G33" s="1" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C34" s="7" t="s">
         <v>99</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>100</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>14</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="9" t="s">
+      <c r="A35" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="B35" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="B35" s="8" t="s">
+      <c r="C35" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="C35" s="10" t="s">
+      <c r="D35" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="10"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="10"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="D35" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E35" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F35" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="G35" s="4" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="9"/>
-      <c r="B36" s="8"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="8"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="8"/>
-      <c r="G36" s="4" t="s">
+    </row>
+    <row r="37" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C37" s="11" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="9" t="s">
+      <c r="D37" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="B37" s="8" t="s">
+      <c r="E37" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="C37" s="10" t="s">
+      <c r="F37" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A38" s="10"/>
+      <c r="B38" s="9"/>
+      <c r="C38" s="11"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="9"/>
+      <c r="G38" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D37" s="8" t="s">
+    </row>
+    <row r="39" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A39" s="10"/>
+      <c r="B39" s="9"/>
+      <c r="C39" s="11"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="9"/>
+      <c r="G39" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="E37" s="9" t="s">
+    </row>
+    <row r="40" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="10"/>
+      <c r="B40" s="9"/>
+      <c r="C40" s="11"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="9"/>
+      <c r="G40" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F37" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="9"/>
-      <c r="B38" s="8"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="8"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="8"/>
-      <c r="G38" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A39" s="9"/>
-      <c r="B39" s="8"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="8"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="8"/>
-      <c r="G39" s="1" t="s">
+    </row>
+    <row r="41" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A41" s="10"/>
+      <c r="B41" s="9"/>
+      <c r="C41" s="11"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="9"/>
+      <c r="G41" s="1" t="s">
         <v>117</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="9"/>
-      <c r="B40" s="8"/>
-      <c r="C40" s="10"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="9"/>
-      <c r="F40" s="8"/>
-      <c r="G40" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A41" s="9"/>
-      <c r="B41" s="8"/>
-      <c r="C41" s="10"/>
-      <c r="D41" s="8"/>
-      <c r="E41" s="9"/>
-      <c r="F41" s="8"/>
-      <c r="G41" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="60">
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="F4:F8"/>
-    <mergeCell ref="F9:F12"/>
-    <mergeCell ref="F13:F15"/>
-    <mergeCell ref="F16:F21"/>
-    <mergeCell ref="A4:A8"/>
-    <mergeCell ref="B4:B8"/>
-    <mergeCell ref="C4:C8"/>
-    <mergeCell ref="D4:D8"/>
-    <mergeCell ref="E4:E8"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="D13:D15"/>
-    <mergeCell ref="E13:E15"/>
-    <mergeCell ref="E9:E12"/>
-    <mergeCell ref="D9:D12"/>
-    <mergeCell ref="C9:C12"/>
-    <mergeCell ref="B9:B12"/>
-    <mergeCell ref="A9:A12"/>
-    <mergeCell ref="F31:F33"/>
-    <mergeCell ref="A16:A21"/>
-    <mergeCell ref="B16:B21"/>
-    <mergeCell ref="C16:C21"/>
-    <mergeCell ref="D16:D21"/>
-    <mergeCell ref="E16:E21"/>
-    <mergeCell ref="E24:E26"/>
-    <mergeCell ref="D24:D26"/>
-    <mergeCell ref="C24:C26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="F37:F41"/>
+    <mergeCell ref="E37:E41"/>
+    <mergeCell ref="D37:D41"/>
+    <mergeCell ref="C37:C41"/>
+    <mergeCell ref="B37:B41"/>
     <mergeCell ref="A37:A41"/>
     <mergeCell ref="D35:D36"/>
     <mergeCell ref="E35:E36"/>
@@ -1622,11 +1712,348 @@
     <mergeCell ref="C31:C33"/>
     <mergeCell ref="D31:D33"/>
     <mergeCell ref="E31:E33"/>
-    <mergeCell ref="F37:F41"/>
-    <mergeCell ref="E37:E41"/>
-    <mergeCell ref="D37:D41"/>
-    <mergeCell ref="C37:C41"/>
-    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="F31:F33"/>
+    <mergeCell ref="A16:A21"/>
+    <mergeCell ref="B16:B21"/>
+    <mergeCell ref="C16:C21"/>
+    <mergeCell ref="D16:D21"/>
+    <mergeCell ref="E16:E21"/>
+    <mergeCell ref="E24:E26"/>
+    <mergeCell ref="D24:D26"/>
+    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="E9:E12"/>
+    <mergeCell ref="D9:D12"/>
+    <mergeCell ref="C9:C12"/>
+    <mergeCell ref="B9:B12"/>
+    <mergeCell ref="A9:A12"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="D13:D15"/>
+    <mergeCell ref="E13:E15"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="A4:A8"/>
+    <mergeCell ref="B4:B8"/>
+    <mergeCell ref="C4:C8"/>
+    <mergeCell ref="D4:D8"/>
+    <mergeCell ref="E4:E8"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="F4:F8"/>
+    <mergeCell ref="F9:F12"/>
+    <mergeCell ref="F13:F15"/>
+    <mergeCell ref="F16:F21"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFB17AF2-F675-49FF-B120-470F5A4D23AB}">
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="34.44140625" customWidth="1"/>
+    <col min="2" max="2" width="16" style="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.21875" customWidth="1"/>
+    <col min="5" max="5" width="16.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="35" t="s">
+        <v>120</v>
+      </c>
+      <c r="C2" s="36">
+        <v>1</v>
+      </c>
+      <c r="D2" s="26"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="13"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="29"/>
+      <c r="B3" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="13"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="29"/>
+      <c r="B4" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="23">
+        <v>4</v>
+      </c>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="13"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="29"/>
+      <c r="B5" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="16">
+        <v>1</v>
+      </c>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="13"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="33"/>
+      <c r="B6" s="31" t="s">
+        <v>123</v>
+      </c>
+      <c r="C6" s="32">
+        <f>SUM(C2:C5)</f>
+        <v>6</v>
+      </c>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="13"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="C7" s="12">
+        <v>1</v>
+      </c>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="13"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="30"/>
+      <c r="B8" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="13"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="30"/>
+      <c r="B9" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="13"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="30"/>
+      <c r="B10" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="34"/>
+      <c r="B11" s="31" t="s">
+        <v>123</v>
+      </c>
+      <c r="C11" s="32">
+        <f>SUM(C7:C10)</f>
+        <v>1</v>
+      </c>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="29" t="s">
+        <v>125</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="29"/>
+      <c r="B13" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="C13" s="21">
+        <v>1</v>
+      </c>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="29"/>
+      <c r="B14" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="29"/>
+      <c r="B15" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="D15" s="13"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="14"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="33"/>
+      <c r="B16" s="31" t="s">
+        <v>123</v>
+      </c>
+      <c r="C16" s="32">
+        <f>SUM(C12:C15)</f>
+        <v>1</v>
+      </c>
+      <c r="D16" s="19"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="14"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="B17" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="D17" s="19"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="14"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="29"/>
+      <c r="B18" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="D18" s="17"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="14"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="29"/>
+      <c r="B19" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C19" s="21">
+        <v>4</v>
+      </c>
+      <c r="D19" s="19"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="14"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="29"/>
+      <c r="B20" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" s="16">
+        <v>1</v>
+      </c>
+      <c r="D20" s="17"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="14"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="33"/>
+      <c r="B21" s="31" t="s">
+        <v>123</v>
+      </c>
+      <c r="C21" s="32">
+        <f>SUM(C17:C20)</f>
+        <v>5</v>
+      </c>
+      <c r="D21" s="17"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="14"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="B22" s="27" t="s">
+        <v>123</v>
+      </c>
+      <c r="C22" s="28">
+        <v>4</v>
+      </c>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A12:A16"/>
+    <mergeCell ref="A17:A21"/>
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="A7:A11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Aagaard, Larson, and classification fixes, apendix start 1-13-2025
</commit_message>
<xml_diff>
--- a/data/BoomBust_Mechanisms.xlsx
+++ b/data/BoomBust_Mechanisms.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f4f5e485ed766aa2/Pictures/Documents/Career/Journal Publications/Manuscripts/Dissertation/boom-bust/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="712" documentId="8_{1B1AAC56-C345-4EC3-95A7-6FD9A5B02C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B2152032-4CBD-4712-BE58-043CEFB140DC}"/>
+  <xr:revisionPtr revIDLastSave="787" documentId="8_{1B1AAC56-C345-4EC3-95A7-6FD9A5B02C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23097938-25DD-4794-9008-AA236724967F}"/>
   <bookViews>
-    <workbookView xWindow="-19320" yWindow="-60" windowWidth="19440" windowHeight="14880" activeTab="1" xr2:uid="{D0698BA0-D8A4-462B-B44D-ABAD27A63A84}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="14016" windowHeight="12336" activeTab="1" xr2:uid="{D0698BA0-D8A4-462B-B44D-ABAD27A63A84}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="130">
   <si>
     <t>Paper</t>
   </si>
@@ -257,9 +257,6 @@
   </si>
   <si>
     <t>Pseudodiaptomus forbesi</t>
-  </si>
-  <si>
-    <t>multiple</t>
   </si>
   <si>
     <t>Aurelia aurita</t>
@@ -445,6 +442,15 @@
   </si>
   <si>
     <t>1) Cold water and drought events preceeded the boom-bust, and large non-native fishes experienced declines during those cold water conditions and drought conditions</t>
+  </si>
+  <si>
+    <t>Acridotheres tristis; Passer domesticus; Garrulax canorus; Lonchura punctulata; Amandava amandava; Sicalis flaveola; Sturnella neglecta; Crithagra mozambica; Geopelia striata; Spilopelia chinensis; Psittacula krameri; Brotogeris versicolurus</t>
+  </si>
+  <si>
+    <t># of time series</t>
+  </si>
+  <si>
+    <t># of species</t>
   </si>
 </sst>
 </file>
@@ -534,7 +540,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -555,90 +561,77 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -655,10 +648,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -998,7 +987,7 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
@@ -1014,7 +1003,7 @@
         <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
@@ -1022,7 +1011,7 @@
         <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1032,21 +1021,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CF18FAA-193E-4ADD-BAC0-7E416D9C0956}">
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.5546875" customWidth="1"/>
     <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.21875" customWidth="1"/>
-    <col min="4" max="4" width="24.109375" customWidth="1"/>
-    <col min="5" max="5" width="17" customWidth="1"/>
-    <col min="6" max="6" width="18.77734375" customWidth="1"/>
-    <col min="7" max="7" width="67.6640625" customWidth="1"/>
-    <col min="8" max="8" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="57.77734375" customWidth="1"/>
+    <col min="4" max="6" width="24.109375" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="8" max="8" width="18.77734375" customWidth="1"/>
+    <col min="9" max="9" width="67.6640625" customWidth="1"/>
+    <col min="10" max="10" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="57.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1060,296 +1049,362 @@
         <v>13</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+      <c r="I1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="30">
+        <v>1</v>
+      </c>
+      <c r="F2" s="30">
+        <v>1</v>
+      </c>
+      <c r="G2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="H2" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="72" x14ac:dyDescent="0.3">
-      <c r="A3" s="10"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="1" t="s">
+    <row r="3" spans="1:9" ht="72" x14ac:dyDescent="0.3">
+      <c r="A3" s="22"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="31">
+        <v>1</v>
+      </c>
+      <c r="F4" s="31">
+        <v>1</v>
+      </c>
+      <c r="G4" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="H4" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="22"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="22"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" s="22"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="31"/>
+      <c r="F7" s="31"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="22"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="31"/>
+      <c r="F8" s="31"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
+      <c r="I8" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" s="31">
+        <v>1</v>
+      </c>
+      <c r="F9" s="31">
+        <v>1</v>
+      </c>
+      <c r="G9" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="H9" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="G4" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="10"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="10"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="10"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="10"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="G9" s="1" t="s">
+      <c r="I9" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="10"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="1" t="s">
+    <row r="10" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="22"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="10"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="1" t="s">
+    <row r="11" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="22"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="21"/>
+      <c r="I11" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="10"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="1" t="s">
+    <row r="12" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="22"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="21"/>
+      <c r="I12" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="10" t="s">
+    <row r="13" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="29">
+        <v>1</v>
+      </c>
+      <c r="F13" s="29">
+        <v>1</v>
+      </c>
+      <c r="G13" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="H13" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="I13" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="1" t="s">
+    <row r="14" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A14" s="22"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="21"/>
+      <c r="I14" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="1" t="s">
+    <row r="15" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A15" s="22"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="21"/>
+      <c r="I15" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="10" t="s">
+    <row r="16" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="23" t="s">
         <v>72</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="E16" s="29">
+        <v>1</v>
+      </c>
+      <c r="F16" s="29">
+        <v>1</v>
+      </c>
+      <c r="G16" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="H16" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="I16" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A17" s="10"/>
-      <c r="B17" s="9"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="1" t="s">
+    <row r="17" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="22"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="21"/>
+      <c r="I17" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="10"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="1" t="s">
+    <row r="18" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="22"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="22"/>
+      <c r="H18" s="21"/>
+      <c r="I18" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="10"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="1" t="s">
+    <row r="19" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A19" s="22"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="21"/>
+      <c r="I19" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="10"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="1" t="s">
+    <row r="20" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="22"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="21"/>
+      <c r="I20" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="10"/>
-      <c r="B21" s="9"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="1" t="s">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" s="22"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="21"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="21"/>
+      <c r="I21" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>50</v>
       </c>
@@ -1357,22 +1412,28 @@
         <v>51</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>73</v>
+        <v>127</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="E22" s="8">
+        <v>12</v>
+      </c>
+      <c r="F22" s="8">
+        <v>12</v>
+      </c>
+      <c r="G22" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="H22" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="G22" s="1" t="s">
+      <c r="I22" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>55</v>
       </c>
@@ -1380,377 +1441,471 @@
         <v>56</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="E23" s="8">
+        <v>1</v>
+      </c>
+      <c r="F23" s="8">
+        <v>1</v>
+      </c>
+      <c r="G23" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="H23" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="G23" s="1" t="s">
+      <c r="I23" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="10" t="s">
+    <row r="24" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A24" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D24" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="E24" s="31">
+        <v>9</v>
+      </c>
+      <c r="F24" s="31">
+        <v>1</v>
+      </c>
+      <c r="G24" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="H24" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="22"/>
+      <c r="B25" s="22"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="31"/>
+      <c r="F25" s="31"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A26" s="22"/>
+      <c r="B26" s="22"/>
+      <c r="C26" s="23"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="22"/>
+      <c r="H26" s="21"/>
+      <c r="I26" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="C27" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="D24" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="E24" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A25" s="10"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A26" s="10"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="C27" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="D27" s="9" t="s">
+      <c r="D27" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="E27" s="29">
+        <v>1</v>
+      </c>
+      <c r="F27" s="29">
+        <v>1</v>
+      </c>
+      <c r="G27" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="F27" s="9" t="s">
+      <c r="H27" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="G27" s="1" t="s">
+      <c r="I27" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A28" s="10"/>
-      <c r="B28" s="9"/>
-      <c r="C28" s="11"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-      <c r="G28" s="1" t="s">
+    <row r="28" spans="1:9" ht="65.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="22"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="21"/>
+      <c r="I28" s="1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="62.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" ht="104.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="C29" s="7" t="s">
         <v>80</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>81</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E29" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="F29" s="6" t="s">
+      <c r="E29" s="8">
+        <v>1</v>
+      </c>
+      <c r="F29" s="8">
+        <v>1</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="H29" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="G29" s="4" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I29" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="118.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B30" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="C30" s="5" t="s">
         <v>87</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>88</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E30" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="F30" s="6" t="s">
+      <c r="E30" s="8">
+        <v>1</v>
+      </c>
+      <c r="F30" s="8">
+        <v>1</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="H30" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="G30" s="4" t="s">
+      <c r="I30" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="22" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="10" t="s">
+      <c r="B31" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="C31" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="C31" s="11" t="s">
+      <c r="D31" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="E31" s="29">
+        <v>1</v>
+      </c>
+      <c r="F31" s="29">
+        <v>1</v>
+      </c>
+      <c r="G31" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="H31" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="I31" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D31" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="E31" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="F31" s="10" t="s">
+    </row>
+    <row r="32" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A32" s="22"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="21"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="I32" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" s="22"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="22"/>
+      <c r="H33" s="22"/>
+      <c r="I33" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B34" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="G31" s="1" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="10"/>
-      <c r="B32" s="9"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="9"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
-      <c r="G32" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" s="10"/>
-      <c r="B33" s="9"/>
-      <c r="C33" s="11"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="4" t="s">
+      <c r="C34" s="7" t="s">
         <v>98</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>99</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E34" s="4" t="s">
+      <c r="E34" s="8">
+        <v>1</v>
+      </c>
+      <c r="F34" s="8">
+        <v>1</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="22" t="s">
         <v>101</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="B35" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="C35" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="D35" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="E35" s="29">
+        <v>2</v>
+      </c>
+      <c r="F35" s="29">
+        <v>1</v>
+      </c>
+      <c r="G35" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="H35" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="G34" s="1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="B35" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="C35" s="11" t="s">
+      <c r="I35" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="22"/>
+      <c r="B36" s="21"/>
+      <c r="C36" s="23"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="29"/>
+      <c r="F36" s="29"/>
+      <c r="G36" s="22"/>
+      <c r="H36" s="21"/>
+      <c r="I36" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D35" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="E35" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="F35" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G35" s="4" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="10"/>
-      <c r="B36" s="9"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="9"/>
-      <c r="G36" s="4" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="10" t="s">
+    </row>
+    <row r="37" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="B37" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="C37" s="23" t="s">
+        <v>106</v>
+      </c>
+      <c r="D37" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="C37" s="11" t="s">
+      <c r="E37" s="29">
+        <v>2</v>
+      </c>
+      <c r="F37" s="29">
+        <v>1</v>
+      </c>
+      <c r="G37" s="22" t="s">
+        <v>113</v>
+      </c>
+      <c r="H37" s="21" t="s">
+        <v>109</v>
+      </c>
+      <c r="I37" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D37" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="E37" s="10" t="s">
+    </row>
+    <row r="38" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A38" s="22"/>
+      <c r="B38" s="21"/>
+      <c r="C38" s="23"/>
+      <c r="D38" s="21"/>
+      <c r="E38" s="29"/>
+      <c r="F38" s="29"/>
+      <c r="G38" s="22"/>
+      <c r="H38" s="21"/>
+      <c r="I38" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A39" s="22"/>
+      <c r="B39" s="21"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="21"/>
+      <c r="E39" s="29"/>
+      <c r="F39" s="29"/>
+      <c r="G39" s="22"/>
+      <c r="H39" s="21"/>
+      <c r="I39" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F37" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="10"/>
-      <c r="B38" s="9"/>
-      <c r="C38" s="11"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="10"/>
-      <c r="F38" s="9"/>
-      <c r="G38" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A39" s="10"/>
-      <c r="B39" s="9"/>
-      <c r="C39" s="11"/>
-      <c r="D39" s="9"/>
-      <c r="E39" s="10"/>
-      <c r="F39" s="9"/>
-      <c r="G39" s="1" t="s">
+    </row>
+    <row r="40" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="22"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="23"/>
+      <c r="D40" s="21"/>
+      <c r="E40" s="29"/>
+      <c r="F40" s="29"/>
+      <c r="G40" s="22"/>
+      <c r="H40" s="21"/>
+      <c r="I40" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="10"/>
-      <c r="B40" s="9"/>
-      <c r="C40" s="11"/>
-      <c r="D40" s="9"/>
-      <c r="E40" s="10"/>
-      <c r="F40" s="9"/>
-      <c r="G40" s="1" t="s">
+    <row r="41" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A41" s="22"/>
+      <c r="B41" s="21"/>
+      <c r="C41" s="23"/>
+      <c r="D41" s="21"/>
+      <c r="E41" s="29"/>
+      <c r="F41" s="29"/>
+      <c r="G41" s="22"/>
+      <c r="H41" s="21"/>
+      <c r="I41" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A41" s="10"/>
-      <c r="B41" s="9"/>
-      <c r="C41" s="11"/>
-      <c r="D41" s="9"/>
-      <c r="E41" s="10"/>
-      <c r="F41" s="9"/>
-      <c r="G41" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="60">
-    <mergeCell ref="F37:F41"/>
-    <mergeCell ref="E37:E41"/>
-    <mergeCell ref="D37:D41"/>
-    <mergeCell ref="C37:C41"/>
-    <mergeCell ref="B37:B41"/>
-    <mergeCell ref="A37:A41"/>
-    <mergeCell ref="D35:D36"/>
+  <mergeCells count="80">
     <mergeCell ref="E35:E36"/>
     <mergeCell ref="F35:F36"/>
-    <mergeCell ref="B24:B26"/>
-    <mergeCell ref="A24:A26"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="E37:E41"/>
+    <mergeCell ref="F37:F41"/>
+    <mergeCell ref="E24:E26"/>
     <mergeCell ref="F24:F26"/>
+    <mergeCell ref="E27:E28"/>
     <mergeCell ref="F27:F28"/>
-    <mergeCell ref="A31:A33"/>
-    <mergeCell ref="B31:B33"/>
-    <mergeCell ref="C31:C33"/>
-    <mergeCell ref="D31:D33"/>
     <mergeCell ref="E31:E33"/>
     <mergeCell ref="F31:F33"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="H4:H8"/>
+    <mergeCell ref="H9:H12"/>
+    <mergeCell ref="H13:H15"/>
+    <mergeCell ref="H16:H21"/>
+    <mergeCell ref="A4:A8"/>
+    <mergeCell ref="B4:B8"/>
+    <mergeCell ref="C4:C8"/>
+    <mergeCell ref="D4:D8"/>
+    <mergeCell ref="G4:G8"/>
+    <mergeCell ref="E4:E8"/>
+    <mergeCell ref="F4:F8"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="D13:D15"/>
+    <mergeCell ref="G13:G15"/>
+    <mergeCell ref="E13:E15"/>
+    <mergeCell ref="F13:F15"/>
+    <mergeCell ref="G9:G12"/>
+    <mergeCell ref="D9:D12"/>
+    <mergeCell ref="C9:C12"/>
+    <mergeCell ref="B9:B12"/>
+    <mergeCell ref="A9:A12"/>
+    <mergeCell ref="E9:E12"/>
+    <mergeCell ref="F9:F12"/>
+    <mergeCell ref="H31:H33"/>
     <mergeCell ref="A16:A21"/>
     <mergeCell ref="B16:B21"/>
     <mergeCell ref="C16:C21"/>
     <mergeCell ref="D16:D21"/>
-    <mergeCell ref="E16:E21"/>
-    <mergeCell ref="E24:E26"/>
+    <mergeCell ref="G16:G21"/>
+    <mergeCell ref="G24:G26"/>
     <mergeCell ref="D24:D26"/>
     <mergeCell ref="C24:C26"/>
     <mergeCell ref="A27:A28"/>
     <mergeCell ref="B27:B28"/>
     <mergeCell ref="C27:C28"/>
     <mergeCell ref="D27:D28"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="E9:E12"/>
-    <mergeCell ref="D9:D12"/>
-    <mergeCell ref="C9:C12"/>
-    <mergeCell ref="B9:B12"/>
-    <mergeCell ref="A9:A12"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="D13:D15"/>
-    <mergeCell ref="E13:E15"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="A4:A8"/>
-    <mergeCell ref="B4:B8"/>
-    <mergeCell ref="C4:C8"/>
-    <mergeCell ref="D4:D8"/>
-    <mergeCell ref="E4:E8"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="F4:F8"/>
-    <mergeCell ref="F9:F12"/>
-    <mergeCell ref="F13:F15"/>
+    <mergeCell ref="G27:G28"/>
+    <mergeCell ref="E16:E21"/>
     <mergeCell ref="F16:F21"/>
+    <mergeCell ref="A37:A41"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="G35:G36"/>
+    <mergeCell ref="H35:H36"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="H24:H26"/>
+    <mergeCell ref="H27:H28"/>
+    <mergeCell ref="A31:A33"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="C31:C33"/>
+    <mergeCell ref="D31:D33"/>
+    <mergeCell ref="G31:G33"/>
+    <mergeCell ref="H37:H41"/>
+    <mergeCell ref="G37:G41"/>
+    <mergeCell ref="D37:D41"/>
+    <mergeCell ref="C37:C41"/>
+    <mergeCell ref="B37:B41"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1762,7 +1917,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34.44140625" customWidth="1"/>
-    <col min="2" max="2" width="16" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" style="14" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.21875" customWidth="1"/>
     <col min="5" max="5" width="16.5546875" bestFit="1" customWidth="1"/>
@@ -1772,281 +1927,239 @@
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="13" t="s">
         <v>3</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" s="35" t="s">
+      <c r="C2" s="20">
+        <v>1</v>
+      </c>
+      <c r="D2" s="11"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="4"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="22"/>
+      <c r="B3" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="C2" s="36">
-        <v>1</v>
-      </c>
-      <c r="D2" s="26"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="13"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="29"/>
-      <c r="B3" s="19" t="s">
-        <v>121</v>
-      </c>
-      <c r="C3" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="13"/>
+      <c r="C3" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="F3" s="4"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="29"/>
-      <c r="B4" s="19" t="s">
+      <c r="A4" s="22"/>
+      <c r="B4" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="23">
+      <c r="C4" s="12">
         <v>4</v>
       </c>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="13"/>
+      <c r="F4" s="4"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="29"/>
-      <c r="B5" s="19" t="s">
+      <c r="A5" s="22"/>
+      <c r="B5" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="16">
-        <v>1</v>
-      </c>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="13"/>
+      <c r="C5" s="8">
+        <v>1</v>
+      </c>
+      <c r="F5" s="4"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="33"/>
-      <c r="B6" s="31" t="s">
-        <v>123</v>
-      </c>
-      <c r="C6" s="32">
+      <c r="A6" s="25"/>
+      <c r="B6" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="C6" s="18">
         <f>SUM(C2:C5)</f>
         <v>6</v>
       </c>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="13"/>
+      <c r="F6" s="4"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="30" t="s">
-        <v>114</v>
-      </c>
-      <c r="B7" s="20" t="s">
+      <c r="A7" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="8">
+        <v>1</v>
+      </c>
+      <c r="F7" s="4"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="27"/>
+      <c r="B8" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="C7" s="12">
-        <v>1</v>
-      </c>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="13"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="30"/>
-      <c r="B8" s="18" t="s">
+      <c r="C8" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="27"/>
+      <c r="B9" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="F9" s="4"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="27"/>
+      <c r="B10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="28"/>
+      <c r="B11" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="C11" s="18">
+        <f>SUM(C7:C10)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="22"/>
+      <c r="B13" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="C13" s="12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="22"/>
+      <c r="B14" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="22"/>
+      <c r="B15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="8"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="25"/>
+      <c r="B16" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="C16" s="18">
+        <f>SUM(C12:C15)</f>
+        <v>1</v>
+      </c>
+      <c r="D16" s="10"/>
+      <c r="E16" s="8"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="C8" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="13"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="30"/>
-      <c r="B9" s="18" t="s">
+      <c r="B17" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="D17" s="10"/>
+      <c r="E17" s="8"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="22"/>
+      <c r="B18" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="D18" s="6"/>
+      <c r="E18" s="8"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="22"/>
+      <c r="B19" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="13"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="30"/>
-      <c r="B10" s="19" t="s">
+      <c r="C19" s="12">
+        <v>4</v>
+      </c>
+      <c r="D19" s="10"/>
+      <c r="E19" s="8"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="22"/>
+      <c r="B20" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="16" t="s">
-        <v>124</v>
-      </c>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="34"/>
-      <c r="B11" s="31" t="s">
-        <v>123</v>
-      </c>
-      <c r="C11" s="32">
-        <f>SUM(C7:C10)</f>
-        <v>1</v>
-      </c>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="29" t="s">
-        <v>125</v>
-      </c>
-      <c r="B12" s="20" t="s">
-        <v>120</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="29"/>
-      <c r="B13" s="18" t="s">
-        <v>121</v>
-      </c>
-      <c r="C13" s="21">
-        <v>1</v>
-      </c>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="29"/>
-      <c r="B14" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="29"/>
-      <c r="B15" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="16" t="s">
-        <v>124</v>
-      </c>
-      <c r="D15" s="13"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="14"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="33"/>
-      <c r="B16" s="31" t="s">
-        <v>123</v>
-      </c>
-      <c r="C16" s="32">
-        <f>SUM(C12:C15)</f>
-        <v>1</v>
-      </c>
-      <c r="D16" s="19"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="14"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="29" t="s">
+      <c r="C20" s="8">
+        <v>1</v>
+      </c>
+      <c r="D20" s="6"/>
+      <c r="E20" s="8"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="25"/>
+      <c r="B21" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="B17" s="20" t="s">
-        <v>120</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="D17" s="19"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="14"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="29"/>
-      <c r="B18" s="18" t="s">
-        <v>121</v>
-      </c>
-      <c r="C18" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="D18" s="17"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="14"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="29"/>
-      <c r="B19" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="C19" s="21">
-        <v>4</v>
-      </c>
-      <c r="D19" s="19"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="14"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="29"/>
-      <c r="B20" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="C20" s="16">
-        <v>1</v>
-      </c>
-      <c r="D20" s="17"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="14"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="33"/>
-      <c r="B21" s="31" t="s">
-        <v>123</v>
-      </c>
-      <c r="C21" s="32">
+      <c r="C21" s="18">
         <f>SUM(C17:C20)</f>
         <v>5</v>
       </c>
-      <c r="D21" s="17"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="14"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="B22" s="27" t="s">
-        <v>123</v>
-      </c>
-      <c r="C22" s="28">
+      <c r="D21" s="6"/>
+      <c r="E21" s="8"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="C22" s="16">
         <v>4</v>
       </c>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Repository Cleanup 01: 6-23-2026
</commit_message>
<xml_diff>
--- a/data/BoomBust_Mechanisms.xlsx
+++ b/data/BoomBust_Mechanisms.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f4f5e485ed766aa2/Pictures/Documents/Career/Journal Publications/Manuscripts/Dissertation/boom-bust/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="787" documentId="8_{1B1AAC56-C345-4EC3-95A7-6FD9A5B02C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23097938-25DD-4794-9008-AA236724967F}"/>
+  <xr:revisionPtr revIDLastSave="808" documentId="8_{1B1AAC56-C345-4EC3-95A7-6FD9A5B02C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E360797-FDA0-41B7-B1CA-46B35DD59692}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="14016" windowHeight="12336" activeTab="1" xr2:uid="{D0698BA0-D8A4-462B-B44D-ABAD27A63A84}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{D0698BA0-D8A4-462B-B44D-ABAD27A63A84}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="132">
   <si>
     <t>Paper</t>
   </si>
@@ -290,9 +290,6 @@
   </si>
   <si>
     <t>The paper has strong evidence, empirical work testing hypothesized mechanism is presented or cited and is expreimentally obtained, observational evidence includes models with drivers and response data that were apriori selected,alternative mechanisms have also been evaluated and ruled out, the suggested mechanisms is very likely the mechanism. Evidence can be demographically tied.</t>
-  </si>
-  <si>
-    <t>The paper  has evidence, empirical work testing hypothesized mechanism is presented or cited but is mostely correlary alternative mechanisms have also been evaluated and ruled out, may have some post hoc modelling with suggested mechansims. The mechanism presented is likely. Mechanism is not demographically tied.</t>
   </si>
   <si>
     <t>Boom means bust: interactons between El Nino Southern Oscillation (ENSO), rainfall and the processes threatening mammal species in arid australia</t>
@@ -452,12 +449,21 @@
   <si>
     <t># of species</t>
   </si>
+  <si>
+    <t>Number of Time series</t>
+  </si>
+  <si>
+    <t>Number of Species</t>
+  </si>
+  <si>
+    <t>The paper has evidence, empirical work testing hypothesized mechanism is presented or cited but is mostely correlary alternative mechanisms have also been evaluated and ruled out, may have some post hoc modelling with suggested mechansims. The mechanism presented is likely. Mechanism is not demographically tied.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -481,6 +487,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -490,7 +509,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -536,11 +555,40 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="dotted">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="dotted">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="dotted">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -568,18 +616,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -601,6 +637,15 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -610,7 +655,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -618,19 +663,50 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -648,6 +724,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1003,7 +1083,7 @@
         <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>84</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
@@ -1026,7 +1106,7 @@
   <cols>
     <col min="1" max="1" width="23.5546875" customWidth="1"/>
     <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.21875" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" customWidth="1"/>
     <col min="4" max="6" width="24.109375" customWidth="1"/>
     <col min="7" max="7" width="17" customWidth="1"/>
     <col min="8" max="8" width="18.77734375" customWidth="1"/>
@@ -1049,10 +1129,10 @@
         <v>13</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>128</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>129</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>2</v>
@@ -1065,28 +1145,28 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="23" t="s">
+      <c r="C2" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="30">
-        <v>1</v>
-      </c>
-      <c r="F2" s="30">
-        <v>1</v>
-      </c>
-      <c r="G2" s="24" t="s">
+      <c r="E2" s="23">
+        <v>1</v>
+      </c>
+      <c r="F2" s="23">
+        <v>1</v>
+      </c>
+      <c r="G2" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="H2" s="24" t="s">
+      <c r="H2" s="19" t="s">
         <v>26</v>
       </c>
       <c r="I2" t="s">
@@ -1094,41 +1174,41 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="72" x14ac:dyDescent="0.3">
-      <c r="A3" s="22"/>
-      <c r="B3" s="21"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
+      <c r="A3" s="21"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
       <c r="I3" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="31">
-        <v>1</v>
-      </c>
-      <c r="F4" s="31">
-        <v>1</v>
-      </c>
-      <c r="G4" s="22" t="s">
+      <c r="E4" s="18">
+        <v>1</v>
+      </c>
+      <c r="F4" s="18">
+        <v>1</v>
+      </c>
+      <c r="G4" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="H4" s="22" t="s">
+      <c r="H4" s="21" t="s">
         <v>76</v>
       </c>
       <c r="I4" s="1" t="s">
@@ -1136,80 +1216,80 @@
       </c>
     </row>
     <row r="5" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="22"/>
-      <c r="B5" s="21"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="31"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
+      <c r="A5" s="21"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
       <c r="I5" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="22"/>
-      <c r="B6" s="21"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
+      <c r="A6" s="21"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
       <c r="I6" s="1" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="22"/>
-      <c r="B7" s="21"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="31"/>
-      <c r="F7" s="31"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
+      <c r="A7" s="21"/>
+      <c r="B7" s="20"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="21"/>
       <c r="I7" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="22"/>
-      <c r="B8" s="21"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="31"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
+      <c r="A8" s="21"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="21"/>
       <c r="I8" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="D9" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="31">
-        <v>1</v>
-      </c>
-      <c r="F9" s="31">
-        <v>1</v>
-      </c>
-      <c r="G9" s="22" t="s">
-        <v>117</v>
-      </c>
-      <c r="H9" s="21" t="s">
+      <c r="E9" s="18">
+        <v>1</v>
+      </c>
+      <c r="F9" s="18">
+        <v>1</v>
+      </c>
+      <c r="G9" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="H9" s="20" t="s">
         <v>77</v>
       </c>
       <c r="I9" s="1" t="s">
@@ -1217,67 +1297,67 @@
       </c>
     </row>
     <row r="10" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="22"/>
-      <c r="B10" s="21"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="31"/>
-      <c r="F10" s="31"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="21"/>
+      <c r="A10" s="21"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="20"/>
       <c r="I10" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="22"/>
-      <c r="B11" s="21"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="31"/>
-      <c r="F11" s="31"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="21"/>
+      <c r="A11" s="21"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="20"/>
       <c r="I11" s="1" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="22"/>
-      <c r="B12" s="21"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="31"/>
-      <c r="F12" s="31"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="21"/>
+      <c r="A12" s="21"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="20"/>
       <c r="I12" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="D13" s="21" t="s">
+      <c r="D13" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="29">
-        <v>1</v>
-      </c>
-      <c r="F13" s="29">
-        <v>1</v>
-      </c>
-      <c r="G13" s="22" t="s">
+      <c r="E13" s="17">
+        <v>1</v>
+      </c>
+      <c r="F13" s="17">
+        <v>1</v>
+      </c>
+      <c r="G13" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="H13" s="21" t="s">
+      <c r="H13" s="20" t="s">
         <v>43</v>
       </c>
       <c r="I13" s="1" t="s">
@@ -1285,54 +1365,54 @@
       </c>
     </row>
     <row r="14" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="22"/>
-      <c r="B14" s="22"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="29"/>
-      <c r="F14" s="29"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="21"/>
+      <c r="A14" s="21"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="20"/>
       <c r="I14" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="22"/>
-      <c r="B15" s="22"/>
-      <c r="C15" s="23"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="29"/>
-      <c r="F15" s="29"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="21"/>
+      <c r="A15" s="21"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="20"/>
       <c r="I15" s="1" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="C16" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="D16" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E16" s="29">
-        <v>1</v>
-      </c>
-      <c r="F16" s="29">
-        <v>1</v>
-      </c>
-      <c r="G16" s="22" t="s">
+      <c r="E16" s="17">
+        <v>1</v>
+      </c>
+      <c r="F16" s="17">
+        <v>1</v>
+      </c>
+      <c r="G16" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="H16" s="21" t="s">
+      <c r="H16" s="20" t="s">
         <v>43</v>
       </c>
       <c r="I16" s="1" t="s">
@@ -1340,79 +1420,79 @@
       </c>
     </row>
     <row r="17" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A17" s="22"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="29"/>
-      <c r="F17" s="29"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="21"/>
+      <c r="A17" s="21"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="21"/>
+      <c r="H17" s="20"/>
       <c r="I17" s="1" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="22"/>
-      <c r="B18" s="21"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="29"/>
-      <c r="F18" s="29"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="21"/>
+      <c r="A18" s="21"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="20"/>
       <c r="I18" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="22"/>
-      <c r="B19" s="21"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="21"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="29"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="21"/>
+      <c r="A19" s="21"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="21"/>
+      <c r="H19" s="20"/>
       <c r="I19" s="1" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="22"/>
-      <c r="B20" s="21"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="29"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="21"/>
+      <c r="A20" s="21"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="21"/>
+      <c r="H20" s="20"/>
       <c r="I20" s="1" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" s="22"/>
-      <c r="B21" s="21"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="29"/>
-      <c r="F21" s="29"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="21"/>
+      <c r="A21" s="21"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="21"/>
+      <c r="H21" s="20"/>
       <c r="I21" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>50</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C22" s="5" t="s">
-        <v>127</v>
+      <c r="C22" s="7" t="s">
+        <v>126</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>52</v>
@@ -1463,28 +1543,28 @@
       </c>
     </row>
     <row r="24" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="B24" s="22" t="s">
+      <c r="B24" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="23" t="s">
+      <c r="C24" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="D24" s="22" t="s">
+      <c r="D24" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="E24" s="31">
+      <c r="E24" s="18">
         <v>9</v>
       </c>
-      <c r="F24" s="31">
-        <v>1</v>
-      </c>
-      <c r="G24" s="22" t="s">
+      <c r="F24" s="18">
+        <v>1</v>
+      </c>
+      <c r="G24" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="H24" s="21" t="s">
+      <c r="H24" s="20" t="s">
         <v>43</v>
       </c>
       <c r="I24" s="1" t="s">
@@ -1492,54 +1572,54 @@
       </c>
     </row>
     <row r="25" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A25" s="22"/>
-      <c r="B25" s="22"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="31"/>
-      <c r="F25" s="31"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="21"/>
+      <c r="A25" s="21"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="21"/>
+      <c r="H25" s="20"/>
       <c r="I25" s="1" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A26" s="22"/>
-      <c r="B26" s="22"/>
-      <c r="C26" s="23"/>
-      <c r="D26" s="22"/>
-      <c r="E26" s="31"/>
-      <c r="F26" s="31"/>
-      <c r="G26" s="22"/>
-      <c r="H26" s="21"/>
+      <c r="A26" s="21"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="21"/>
+      <c r="H26" s="20"/>
       <c r="I26" s="1" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="B27" s="21" t="s">
+      <c r="B27" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C27" s="23" t="s">
+      <c r="C27" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="D27" s="21" t="s">
+      <c r="D27" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E27" s="29">
-        <v>1</v>
-      </c>
-      <c r="F27" s="29">
-        <v>1</v>
-      </c>
-      <c r="G27" s="21" t="s">
+      <c r="E27" s="17">
+        <v>1</v>
+      </c>
+      <c r="F27" s="17">
+        <v>1</v>
+      </c>
+      <c r="G27" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="H27" s="21" t="s">
+      <c r="H27" s="20" t="s">
         <v>26</v>
       </c>
       <c r="I27" s="1" t="s">
@@ -1547,14 +1627,14 @@
       </c>
     </row>
     <row r="28" spans="1:9" ht="65.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="22"/>
-      <c r="B28" s="21"/>
-      <c r="C28" s="23"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="29"/>
-      <c r="F28" s="29"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="21"/>
+      <c r="A28" s="21"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="20"/>
+      <c r="H28" s="20"/>
       <c r="I28" s="1" t="s">
         <v>66</v>
       </c>
@@ -1579,7 +1659,7 @@
         <v>1</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H29" s="6" t="s">
         <v>43</v>
@@ -1590,13 +1670,13 @@
     </row>
     <row r="30" spans="1:9" ht="118.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B30" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="C30" s="5" t="s">
         <v>86</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>87</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>14</v>
@@ -1608,79 +1688,79 @@
         <v>1</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H30" s="6" t="s">
         <v>43</v>
       </c>
       <c r="I30" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="21" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="31" spans="1:9" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="22" t="s">
+      <c r="B31" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="B31" s="21" t="s">
+      <c r="C31" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="C31" s="23" t="s">
+      <c r="D31" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="E31" s="17">
+        <v>1</v>
+      </c>
+      <c r="F31" s="17">
+        <v>1</v>
+      </c>
+      <c r="G31" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="H31" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="I31" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D31" s="21" t="s">
-        <v>14</v>
-      </c>
-      <c r="E31" s="29">
-        <v>1</v>
-      </c>
-      <c r="F31" s="29">
-        <v>1</v>
-      </c>
-      <c r="G31" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="H31" s="22" t="s">
-        <v>95</v>
-      </c>
-      <c r="I31" s="1" t="s">
+    </row>
+    <row r="32" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A32" s="21"/>
+      <c r="B32" s="20"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="20"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
+      <c r="I32" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="22"/>
-      <c r="B32" s="21"/>
-      <c r="C32" s="23"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="29"/>
-      <c r="F32" s="29"/>
-      <c r="G32" s="22"/>
-      <c r="H32" s="22"/>
-      <c r="I32" s="1" t="s">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" s="21"/>
+      <c r="B33" s="20"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="21"/>
+      <c r="H33" s="21"/>
+      <c r="I33" s="1" t="s">
         <v>93</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" s="22"/>
-      <c r="B33" s="21"/>
-      <c r="C33" s="23"/>
-      <c r="D33" s="21"/>
-      <c r="E33" s="29"/>
-      <c r="F33" s="29"/>
-      <c r="G33" s="22"/>
-      <c r="H33" s="22"/>
-      <c r="I33" s="1" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C34" s="7" t="s">
         <v>97</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>98</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>14</v>
@@ -1692,183 +1772,161 @@
         <v>1</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H34" s="4" t="s">
         <v>26</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="22" t="s">
+      <c r="A35" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="B35" s="20" t="s">
         <v>101</v>
       </c>
-      <c r="B35" s="21" t="s">
+      <c r="C35" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="C35" s="23" t="s">
+      <c r="D35" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="E35" s="17">
+        <v>2</v>
+      </c>
+      <c r="F35" s="17">
+        <v>1</v>
+      </c>
+      <c r="G35" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="H35" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="21"/>
+      <c r="B36" s="20"/>
+      <c r="C36" s="22"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="21"/>
+      <c r="H36" s="20"/>
+      <c r="I36" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="D35" s="21" t="s">
-        <v>14</v>
-      </c>
-      <c r="E35" s="29">
+    </row>
+    <row r="37" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="21" t="s">
+        <v>109</v>
+      </c>
+      <c r="B37" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="C37" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="D37" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="E37" s="17">
         <v>2</v>
       </c>
-      <c r="F35" s="29">
-        <v>1</v>
-      </c>
-      <c r="G35" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="H35" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="I35" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="22"/>
-      <c r="B36" s="21"/>
-      <c r="C36" s="23"/>
-      <c r="D36" s="21"/>
-      <c r="E36" s="29"/>
-      <c r="F36" s="29"/>
-      <c r="G36" s="22"/>
-      <c r="H36" s="21"/>
-      <c r="I36" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="22" t="s">
-        <v>110</v>
-      </c>
-      <c r="B37" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="C37" s="23" t="s">
+      <c r="F37" s="17">
+        <v>1</v>
+      </c>
+      <c r="G37" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="H37" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="I37" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D37" s="21" t="s">
-        <v>112</v>
-      </c>
-      <c r="E37" s="29">
-        <v>2</v>
-      </c>
-      <c r="F37" s="29">
-        <v>1</v>
-      </c>
-      <c r="G37" s="22" t="s">
+    </row>
+    <row r="38" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A38" s="21"/>
+      <c r="B38" s="20"/>
+      <c r="C38" s="22"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="21"/>
+      <c r="H38" s="20"/>
+      <c r="I38" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A39" s="21"/>
+      <c r="B39" s="20"/>
+      <c r="C39" s="22"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="17"/>
+      <c r="F39" s="17"/>
+      <c r="G39" s="21"/>
+      <c r="H39" s="20"/>
+      <c r="I39" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="H37" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="I37" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="22"/>
-      <c r="B38" s="21"/>
-      <c r="C38" s="23"/>
-      <c r="D38" s="21"/>
-      <c r="E38" s="29"/>
-      <c r="F38" s="29"/>
-      <c r="G38" s="22"/>
-      <c r="H38" s="21"/>
-      <c r="I38" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A39" s="22"/>
-      <c r="B39" s="21"/>
-      <c r="C39" s="23"/>
-      <c r="D39" s="21"/>
-      <c r="E39" s="29"/>
-      <c r="F39" s="29"/>
-      <c r="G39" s="22"/>
-      <c r="H39" s="21"/>
-      <c r="I39" s="1" t="s">
+    </row>
+    <row r="40" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="21"/>
+      <c r="B40" s="20"/>
+      <c r="C40" s="22"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="17"/>
+      <c r="F40" s="17"/>
+      <c r="G40" s="21"/>
+      <c r="H40" s="20"/>
+      <c r="I40" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="22"/>
-      <c r="B40" s="21"/>
-      <c r="C40" s="23"/>
-      <c r="D40" s="21"/>
-      <c r="E40" s="29"/>
-      <c r="F40" s="29"/>
-      <c r="G40" s="22"/>
-      <c r="H40" s="21"/>
-      <c r="I40" s="1" t="s">
+    <row r="41" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A41" s="21"/>
+      <c r="B41" s="20"/>
+      <c r="C41" s="22"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="17"/>
+      <c r="F41" s="17"/>
+      <c r="G41" s="21"/>
+      <c r="H41" s="20"/>
+      <c r="I41" s="1" t="s">
         <v>115</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A41" s="22"/>
-      <c r="B41" s="21"/>
-      <c r="C41" s="23"/>
-      <c r="D41" s="21"/>
-      <c r="E41" s="29"/>
-      <c r="F41" s="29"/>
-      <c r="G41" s="22"/>
-      <c r="H41" s="21"/>
-      <c r="I41" s="1" t="s">
-        <v>116</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="80">
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="E37:E41"/>
-    <mergeCell ref="F37:F41"/>
-    <mergeCell ref="E24:E26"/>
-    <mergeCell ref="F24:F26"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="E31:E33"/>
-    <mergeCell ref="F31:F33"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="H4:H8"/>
-    <mergeCell ref="H9:H12"/>
-    <mergeCell ref="H13:H15"/>
-    <mergeCell ref="H16:H21"/>
-    <mergeCell ref="A4:A8"/>
-    <mergeCell ref="B4:B8"/>
-    <mergeCell ref="C4:C8"/>
-    <mergeCell ref="D4:D8"/>
-    <mergeCell ref="G4:G8"/>
-    <mergeCell ref="E4:E8"/>
-    <mergeCell ref="F4:F8"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="D13:D15"/>
-    <mergeCell ref="G13:G15"/>
-    <mergeCell ref="E13:E15"/>
-    <mergeCell ref="F13:F15"/>
-    <mergeCell ref="G9:G12"/>
-    <mergeCell ref="D9:D12"/>
-    <mergeCell ref="C9:C12"/>
-    <mergeCell ref="B9:B12"/>
-    <mergeCell ref="A9:A12"/>
-    <mergeCell ref="E9:E12"/>
-    <mergeCell ref="F9:F12"/>
+    <mergeCell ref="H37:H41"/>
+    <mergeCell ref="G37:G41"/>
+    <mergeCell ref="D37:D41"/>
+    <mergeCell ref="C37:C41"/>
+    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="A37:A41"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="G35:G36"/>
+    <mergeCell ref="H35:H36"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="H24:H26"/>
+    <mergeCell ref="H27:H28"/>
+    <mergeCell ref="A31:A33"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="C31:C33"/>
+    <mergeCell ref="D31:D33"/>
+    <mergeCell ref="G31:G33"/>
     <mergeCell ref="H31:H33"/>
     <mergeCell ref="A16:A21"/>
     <mergeCell ref="B16:B21"/>
@@ -1885,27 +1943,49 @@
     <mergeCell ref="G27:G28"/>
     <mergeCell ref="E16:E21"/>
     <mergeCell ref="F16:F21"/>
-    <mergeCell ref="A37:A41"/>
-    <mergeCell ref="D35:D36"/>
-    <mergeCell ref="G35:G36"/>
-    <mergeCell ref="H35:H36"/>
-    <mergeCell ref="B24:B26"/>
-    <mergeCell ref="A24:A26"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="H24:H26"/>
-    <mergeCell ref="H27:H28"/>
-    <mergeCell ref="A31:A33"/>
-    <mergeCell ref="B31:B33"/>
-    <mergeCell ref="C31:C33"/>
-    <mergeCell ref="D31:D33"/>
-    <mergeCell ref="G31:G33"/>
-    <mergeCell ref="H37:H41"/>
-    <mergeCell ref="G37:G41"/>
-    <mergeCell ref="D37:D41"/>
-    <mergeCell ref="C37:C41"/>
-    <mergeCell ref="B37:B41"/>
+    <mergeCell ref="G9:G12"/>
+    <mergeCell ref="D9:D12"/>
+    <mergeCell ref="C9:C12"/>
+    <mergeCell ref="B9:B12"/>
+    <mergeCell ref="A9:A12"/>
+    <mergeCell ref="E9:E12"/>
+    <mergeCell ref="F9:F12"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="D13:D15"/>
+    <mergeCell ref="G13:G15"/>
+    <mergeCell ref="E13:E15"/>
+    <mergeCell ref="F13:F15"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="A4:A8"/>
+    <mergeCell ref="B4:B8"/>
+    <mergeCell ref="C4:C8"/>
+    <mergeCell ref="D4:D8"/>
+    <mergeCell ref="G4:G8"/>
+    <mergeCell ref="E4:E8"/>
+    <mergeCell ref="F4:F8"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="H4:H8"/>
+    <mergeCell ref="H9:H12"/>
+    <mergeCell ref="H13:H15"/>
+    <mergeCell ref="H16:H21"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="E37:E41"/>
+    <mergeCell ref="F37:F41"/>
+    <mergeCell ref="E24:E26"/>
+    <mergeCell ref="F24:F26"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="E31:E33"/>
+    <mergeCell ref="F31:F33"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1917,248 +1997,364 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34.44140625" customWidth="1"/>
-    <col min="2" max="2" width="16" style="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" style="10" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.21875" customWidth="1"/>
     <col min="5" max="5" width="16.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="35" t="s">
+        <v>117</v>
+      </c>
+      <c r="D1" t="s">
+        <v>129</v>
+      </c>
+      <c r="E1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="15" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="26" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" s="19" t="s">
+      <c r="C2" s="16">
+        <v>1</v>
+      </c>
+      <c r="D2" s="37">
+        <v>1</v>
+      </c>
+      <c r="E2" s="37">
+        <v>1</v>
+      </c>
+      <c r="F2" s="4"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="27"/>
+      <c r="B3" s="28" t="s">
         <v>119</v>
       </c>
-      <c r="C2" s="20">
-        <v>1</v>
-      </c>
-      <c r="D2" s="11"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="4"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="22"/>
-      <c r="B3" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>123</v>
+      <c r="C3" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="D3" s="30" t="s">
+        <v>122</v>
+      </c>
+      <c r="E3" s="30" t="s">
+        <v>122</v>
       </c>
       <c r="F3" s="4"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="22"/>
-      <c r="B4" s="10" t="s">
+      <c r="A4" s="27"/>
+      <c r="B4" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="29">
         <v>4</v>
       </c>
+      <c r="D4" s="30">
+        <v>12</v>
+      </c>
+      <c r="E4" s="30">
+        <v>4</v>
+      </c>
       <c r="F4" s="4"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="22"/>
-      <c r="B5" s="10" t="s">
+      <c r="A5" s="27"/>
+      <c r="B5" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="31">
+        <v>1</v>
+      </c>
+      <c r="D5" s="30">
+        <v>2</v>
+      </c>
+      <c r="E5" s="30">
         <v>1</v>
       </c>
       <c r="F5" s="4"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="25"/>
-      <c r="B6" s="17" t="s">
-        <v>122</v>
-      </c>
-      <c r="C6" s="18">
+      <c r="A6" s="24"/>
+      <c r="B6" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="C6" s="14">
         <f>SUM(C2:C5)</f>
         <v>6</v>
       </c>
+      <c r="D6" s="38">
+        <v>15</v>
+      </c>
+      <c r="E6" s="39">
+        <v>6</v>
+      </c>
       <c r="F6" s="4"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="27" t="s">
-        <v>113</v>
-      </c>
-      <c r="B7" s="11" t="s">
+      <c r="A7" s="32" t="s">
+        <v>112</v>
+      </c>
+      <c r="B7" s="33" t="s">
+        <v>118</v>
+      </c>
+      <c r="C7" s="31">
+        <v>1</v>
+      </c>
+      <c r="D7" s="30">
+        <v>2</v>
+      </c>
+      <c r="E7" s="40">
+        <v>1</v>
+      </c>
+      <c r="F7" s="4"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="32"/>
+      <c r="B8" s="28" t="s">
         <v>119</v>
       </c>
-      <c r="C7" s="8">
-        <v>1</v>
-      </c>
-      <c r="F7" s="4"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="27"/>
-      <c r="B8" s="10" t="s">
+      <c r="C8" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="D8" s="30" t="s">
+        <v>122</v>
+      </c>
+      <c r="E8" s="30" t="s">
+        <v>122</v>
+      </c>
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="32"/>
+      <c r="B9" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>122</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>122</v>
+      </c>
+      <c r="F9" s="4"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="32"/>
+      <c r="B10" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="31" t="s">
+        <v>122</v>
+      </c>
+      <c r="D10" s="30" t="s">
+        <v>122</v>
+      </c>
+      <c r="E10" s="30" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="26"/>
+      <c r="B11" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="C11" s="14">
+        <f>SUM(C7:C10)</f>
+        <v>1</v>
+      </c>
+      <c r="D11" s="39">
+        <v>2</v>
+      </c>
+      <c r="E11" s="38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="27" t="s">
+        <v>123</v>
+      </c>
+      <c r="B12" s="33" t="s">
+        <v>118</v>
+      </c>
+      <c r="C12" s="31" t="s">
+        <v>122</v>
+      </c>
+      <c r="D12" s="40" t="s">
+        <v>122</v>
+      </c>
+      <c r="E12" s="30" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="27"/>
+      <c r="B13" s="28" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" s="29">
+        <v>1</v>
+      </c>
+      <c r="D13" s="30">
+        <v>1</v>
+      </c>
+      <c r="E13" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="27"/>
+      <c r="B14" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="D14" s="30" t="s">
+        <v>122</v>
+      </c>
+      <c r="E14" s="30" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="27"/>
+      <c r="B15" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="31" t="s">
+        <v>122</v>
+      </c>
+      <c r="D15" s="30" t="s">
+        <v>122</v>
+      </c>
+      <c r="E15" s="30" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="24"/>
+      <c r="B16" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="C16" s="14">
+        <f>SUM(C12:C15)</f>
+        <v>1</v>
+      </c>
+      <c r="D16" s="39">
+        <v>1</v>
+      </c>
+      <c r="E16" s="39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="27" t="s">
         <v>120</v>
       </c>
-      <c r="C8" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="F8" s="4"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="27"/>
-      <c r="B9" s="10" t="s">
+      <c r="B17" s="33" t="s">
+        <v>118</v>
+      </c>
+      <c r="C17" s="31" t="s">
+        <v>122</v>
+      </c>
+      <c r="D17" s="40" t="s">
+        <v>122</v>
+      </c>
+      <c r="E17" s="40" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="27"/>
+      <c r="B18" s="28" t="s">
+        <v>119</v>
+      </c>
+      <c r="C18" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="D18" s="30" t="s">
+        <v>122</v>
+      </c>
+      <c r="E18" s="30" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="27"/>
+      <c r="B19" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="F9" s="4"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="27"/>
-      <c r="B10" s="10" t="s">
+      <c r="C19" s="29">
+        <v>4</v>
+      </c>
+      <c r="D19" s="30">
+        <v>2</v>
+      </c>
+      <c r="E19" s="30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="27"/>
+      <c r="B20" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="28"/>
-      <c r="B11" s="17" t="s">
-        <v>122</v>
-      </c>
-      <c r="C11" s="18">
-        <f>SUM(C7:C10)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="22" t="s">
-        <v>124</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="22"/>
-      <c r="B13" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="C13" s="12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="22"/>
-      <c r="B14" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="22"/>
-      <c r="B15" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="D15" s="4"/>
-      <c r="E15" s="8"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="25"/>
-      <c r="B16" s="17" t="s">
-        <v>122</v>
-      </c>
-      <c r="C16" s="18">
-        <f>SUM(C12:C15)</f>
-        <v>1</v>
-      </c>
-      <c r="D16" s="10"/>
-      <c r="E16" s="8"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="22" t="s">
+      <c r="C20" s="31">
+        <v>1</v>
+      </c>
+      <c r="D20" s="30">
+        <v>1</v>
+      </c>
+      <c r="E20" s="30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="24"/>
+      <c r="B21" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="B17" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="D17" s="10"/>
-      <c r="E17" s="8"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="22"/>
-      <c r="B18" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="D18" s="6"/>
-      <c r="E18" s="8"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="22"/>
-      <c r="B19" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C19" s="12">
-        <v>4</v>
-      </c>
-      <c r="D19" s="10"/>
-      <c r="E19" s="8"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="22"/>
-      <c r="B20" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="C20" s="8">
-        <v>1</v>
-      </c>
-      <c r="D20" s="6"/>
-      <c r="E20" s="8"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="25"/>
-      <c r="B21" s="17" t="s">
-        <v>122</v>
-      </c>
-      <c r="C21" s="18">
+      <c r="C21" s="14">
         <f>SUM(C17:C20)</f>
         <v>5</v>
       </c>
-      <c r="D21" s="6"/>
-      <c r="E21" s="8"/>
+      <c r="D21" s="39">
+        <v>3</v>
+      </c>
+      <c r="E21" s="38">
+        <v>3</v>
+      </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="C22" s="16">
+        <v>124</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="C22" s="12">
         <v>4</v>
+      </c>
+      <c r="D22" s="41">
+        <v>15</v>
+      </c>
+      <c r="E22" s="34">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>